<commit_message>
added sort 0 and one problem
</commit_message>
<xml_diff>
--- a/out/production/DSA-2024/FINAL450.xlsx
+++ b/out/production/DSA-2024/FINAL450.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DSA-The-Master-Piece-\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A14BBC43-8E34-4031-898E-C899AFD4A220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -442,7 +448,7 @@
     <t>Write a program to Delete loop in a linked list.</t>
   </si>
   <si>
-    <t xml:space="preserve">Find the starting point of the loop. </t>
+    <t>Find the starting point of the loop. </t>
   </si>
   <si>
     <t>Remove Duplicates in a sorted Linked List.</t>
@@ -1222,7 +1228,7 @@
     <t>Program for nth Catalan Number</t>
   </si>
   <si>
-    <t xml:space="preserve">Matrix Chain Multiplication </t>
+    <t>Matrix Chain Multiplication </t>
   </si>
   <si>
     <t>Edit Distance</t>
@@ -1420,9 +1426,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1507,49 +1512,52 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="12">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1560,10 +1568,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -1601,71 +1609,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1693,7 +1701,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1716,11 +1724,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1729,13 +1737,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1745,7 +1753,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1754,7 +1762,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1763,7 +1771,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1771,10 +1779,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1839,38 +1847,38 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C481"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="10" width="28.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="123.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="10" width="27.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="28.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="123" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.5703125" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="29.25">
+    <row r="1" spans="1:3" ht="29.25" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:3" ht="19.5" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="4"/>
       <c r="C3" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="23.25">
+    <row r="4" spans="1:3" ht="23.25" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -1881,14 +1889,14 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:3" ht="18.75" customHeight="1">
       <c r="A5" s="1"/>
       <c r="B5" s="4"/>
       <c r="C5" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="23.25">
+    <row r="6" spans="1:3" ht="23.25" customHeight="1">
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
@@ -1899,7 +1907,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="23.25">
+    <row r="7" spans="1:3" ht="23.25" customHeight="1">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
@@ -1910,7 +1918,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="23.25">
+    <row r="8" spans="1:3" ht="23.25" customHeight="1">
       <c r="A8" s="7" t="s">
         <v>6</v>
       </c>
@@ -1918,10 +1926,10 @@
         <v>10</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="23.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="23.25" customHeight="1">
       <c r="A9" s="7" t="s">
         <v>6</v>
       </c>
@@ -1929,10 +1937,10 @@
         <v>11</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="23.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="23.25" customHeight="1">
       <c r="A10" s="7" t="s">
         <v>6</v>
       </c>
@@ -1943,7 +1951,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="23.25">
+    <row r="11" spans="1:3" ht="23.25" customHeight="1">
       <c r="A11" s="7" t="s">
         <v>6</v>
       </c>
@@ -1954,7 +1962,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="23.25">
+    <row r="12" spans="1:3" ht="23.25" customHeight="1">
       <c r="A12" s="7" t="s">
         <v>6</v>
       </c>
@@ -1965,7 +1973,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="23.25">
+    <row r="13" spans="1:3" ht="23.25" customHeight="1">
       <c r="A13" s="7" t="s">
         <v>6</v>
       </c>
@@ -1973,10 +1981,10 @@
         <v>15</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="23.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="23.25" customHeight="1">
       <c r="A14" s="7" t="s">
         <v>6</v>
       </c>
@@ -1984,10 +1992,10 @@
         <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="23.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="23.25" customHeight="1">
       <c r="A15" s="7" t="s">
         <v>6</v>
       </c>
@@ -1998,7 +2006,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="23.25">
+    <row r="16" spans="1:3" ht="23.25" customHeight="1">
       <c r="A16" s="7" t="s">
         <v>6</v>
       </c>
@@ -2006,10 +2014,10 @@
         <v>18</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="23.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="23.25" customHeight="1">
       <c r="A17" s="7" t="s">
         <v>6</v>
       </c>
@@ -2020,7 +2028,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="24.75">
+    <row r="18" spans="1:3" ht="24.75" customHeight="1">
       <c r="A18" s="7" t="s">
         <v>6</v>
       </c>
@@ -2028,10 +2036,10 @@
         <v>20</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="24.75">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="24.75" customHeight="1">
       <c r="A19" s="7" t="s">
         <v>6</v>
       </c>
@@ -2042,7 +2050,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="24.75">
+    <row r="20" spans="1:3" ht="24.75" customHeight="1">
       <c r="A20" s="7" t="s">
         <v>6</v>
       </c>
@@ -2053,7 +2061,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="24.75">
+    <row r="21" spans="1:3" ht="24.75" customHeight="1">
       <c r="A21" s="7" t="s">
         <v>6</v>
       </c>
@@ -2064,7 +2072,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="24.75">
+    <row r="22" spans="1:3" ht="24.75" customHeight="1">
       <c r="A22" s="7" t="s">
         <v>6</v>
       </c>
@@ -2075,7 +2083,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="24.75">
+    <row r="23" spans="1:3" ht="24.75" customHeight="1">
       <c r="A23" s="7" t="s">
         <v>6</v>
       </c>
@@ -2086,7 +2094,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="24.75">
+    <row r="24" spans="1:3" ht="24.75" customHeight="1">
       <c r="A24" s="7" t="s">
         <v>6</v>
       </c>
@@ -2097,7 +2105,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="24.75">
+    <row r="25" spans="1:3" ht="24.75" customHeight="1">
       <c r="A25" s="7" t="s">
         <v>6</v>
       </c>
@@ -2108,7 +2116,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="24.75">
+    <row r="26" spans="1:3" ht="24.75" customHeight="1">
       <c r="A26" s="7" t="s">
         <v>6</v>
       </c>
@@ -2119,7 +2127,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="24.75">
+    <row r="27" spans="1:3" ht="24.75" customHeight="1">
       <c r="A27" s="7" t="s">
         <v>6</v>
       </c>
@@ -2130,7 +2138,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="24.75">
+    <row r="28" spans="1:3" ht="24.75" customHeight="1">
       <c r="A28" s="7" t="s">
         <v>6</v>
       </c>
@@ -2141,7 +2149,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="24.75">
+    <row r="29" spans="1:3" ht="24.75" customHeight="1">
       <c r="A29" s="7" t="s">
         <v>6</v>
       </c>
@@ -2152,7 +2160,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="24.75">
+    <row r="30" spans="1:3" ht="24.75" customHeight="1">
       <c r="A30" s="7" t="s">
         <v>6</v>
       </c>
@@ -2163,7 +2171,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25">
+    <row r="31" spans="1:3" ht="17.25" customHeight="1">
       <c r="A31" s="7" t="s">
         <v>6</v>
       </c>
@@ -2174,7 +2182,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="17.25">
+    <row r="32" spans="1:3" ht="17.25" customHeight="1">
       <c r="A32" s="7" t="s">
         <v>6</v>
       </c>
@@ -2185,7 +2193,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="17.25">
+    <row r="33" spans="1:3" ht="17.25" customHeight="1">
       <c r="A33" s="7" t="s">
         <v>6</v>
       </c>
@@ -2196,7 +2204,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="17.25">
+    <row r="34" spans="1:3" ht="17.25" customHeight="1">
       <c r="A34" s="7" t="s">
         <v>6</v>
       </c>
@@ -2207,7 +2215,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="17.25">
+    <row r="35" spans="1:3" ht="17.25" customHeight="1">
       <c r="A35" s="7" t="s">
         <v>6</v>
       </c>
@@ -2218,7 +2226,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="17.25">
+    <row r="36" spans="1:3" ht="17.25" customHeight="1">
       <c r="A36" s="7" t="s">
         <v>6</v>
       </c>
@@ -2229,7 +2237,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="23.25">
+    <row r="37" spans="1:3" ht="23.25" customHeight="1">
       <c r="A37" s="7" t="s">
         <v>6</v>
       </c>
@@ -2240,7 +2248,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="23.25">
+    <row r="38" spans="1:3" ht="23.25" customHeight="1">
       <c r="A38" s="7" t="s">
         <v>6</v>
       </c>
@@ -2251,7 +2259,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="23.25">
+    <row r="39" spans="1:3" ht="23.25" customHeight="1">
       <c r="A39" s="7" t="s">
         <v>6</v>
       </c>
@@ -2262,7 +2270,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="23.25">
+    <row r="40" spans="1:3" ht="23.25" customHeight="1">
       <c r="A40" s="7" t="s">
         <v>6</v>
       </c>
@@ -2273,7 +2281,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="23.25">
+    <row r="41" spans="1:3" ht="23.25" customHeight="1">
       <c r="A41" s="7" t="s">
         <v>6</v>
       </c>
@@ -2284,21 +2292,21 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="23.25">
+    <row r="42" spans="1:3" ht="23.25" customHeight="1">
       <c r="A42" s="1"/>
       <c r="B42" s="9"/>
       <c r="C42" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="23.25">
+    <row r="43" spans="1:3" ht="23.25" customHeight="1">
       <c r="A43" s="7"/>
       <c r="B43" s="9"/>
       <c r="C43" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="23.25">
+    <row r="44" spans="1:3" ht="23.25" customHeight="1">
       <c r="A44" s="7" t="s">
         <v>44</v>
       </c>
@@ -2309,7 +2317,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="23.25">
+    <row r="45" spans="1:3" ht="23.25" customHeight="1">
       <c r="A45" s="7" t="s">
         <v>44</v>
       </c>
@@ -2320,7 +2328,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="23.25">
+    <row r="46" spans="1:3" ht="23.25" customHeight="1">
       <c r="A46" s="7" t="s">
         <v>44</v>
       </c>
@@ -2331,7 +2339,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="23.25">
+    <row r="47" spans="1:3" ht="23.25" customHeight="1">
       <c r="A47" s="7" t="s">
         <v>44</v>
       </c>
@@ -2342,7 +2350,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="23.25">
+    <row r="48" spans="1:3" ht="23.25" customHeight="1">
       <c r="A48" s="7" t="s">
         <v>44</v>
       </c>
@@ -2353,7 +2361,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="23.25">
+    <row r="49" spans="1:3" ht="23.25" customHeight="1">
       <c r="A49" s="7" t="s">
         <v>44</v>
       </c>
@@ -2364,7 +2372,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="23.25">
+    <row r="50" spans="1:3" ht="23.25" customHeight="1">
       <c r="A50" s="7" t="s">
         <v>44</v>
       </c>
@@ -2375,7 +2383,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="23.25">
+    <row r="51" spans="1:3" ht="23.25" customHeight="1">
       <c r="A51" s="7" t="s">
         <v>44</v>
       </c>
@@ -2386,7 +2394,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="23.25">
+    <row r="52" spans="1:3" ht="23.25" customHeight="1">
       <c r="A52" s="7" t="s">
         <v>44</v>
       </c>
@@ -2397,7 +2405,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="23.25">
+    <row r="53" spans="1:3" ht="23.25" customHeight="1">
       <c r="A53" s="7" t="s">
         <v>44</v>
       </c>
@@ -2408,17 +2416,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
+    <row r="54" spans="1:3" ht="18.75" customHeight="1">
       <c r="A54" s="1"/>
       <c r="B54" s="4"/>
       <c r="C54" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="23.25">
+    <row r="55" spans="1:3" ht="23.25" customHeight="1">
       <c r="A55" s="7"/>
       <c r="B55" s="9"/>
       <c r="C55" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="23.25">
+    <row r="56" spans="1:3" ht="23.25" customHeight="1">
       <c r="A56" s="7" t="s">
         <v>55</v>
       </c>
@@ -2429,7 +2437,7 @@
         <v>57</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="23.25">
+    <row r="57" spans="1:3" ht="23.25" customHeight="1">
       <c r="A57" s="7" t="s">
         <v>55</v>
       </c>
@@ -2440,7 +2448,7 @@
         <v>57</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="23.25">
+    <row r="58" spans="1:3" ht="23.25" customHeight="1">
       <c r="A58" s="7" t="s">
         <v>55</v>
       </c>
@@ -2451,7 +2459,7 @@
         <v>57</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="23.25">
+    <row r="59" spans="1:3" ht="23.25" customHeight="1">
       <c r="A59" s="7" t="s">
         <v>55</v>
       </c>
@@ -2462,7 +2470,7 @@
         <v>57</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="23.25">
+    <row r="60" spans="1:3" ht="23.25" customHeight="1">
       <c r="A60" s="7" t="s">
         <v>55</v>
       </c>
@@ -2473,7 +2481,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="17.25">
+    <row r="61" spans="1:3" ht="17.25" customHeight="1">
       <c r="A61" s="7" t="s">
         <v>55</v>
       </c>
@@ -2484,7 +2492,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="17.25">
+    <row r="62" spans="1:3" ht="17.25" customHeight="1">
       <c r="A62" s="7" t="s">
         <v>55</v>
       </c>
@@ -2495,7 +2503,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="17.25">
+    <row r="63" spans="1:3" ht="17.25" customHeight="1">
       <c r="A63" s="7" t="s">
         <v>55</v>
       </c>
@@ -2506,7 +2514,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="17.25">
+    <row r="64" spans="1:3" ht="17.25" customHeight="1">
       <c r="A64" s="7" t="s">
         <v>55</v>
       </c>
@@ -2517,7 +2525,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="17.25">
+    <row r="65" spans="1:3" ht="17.25" customHeight="1">
       <c r="A65" s="7" t="s">
         <v>55</v>
       </c>
@@ -2528,7 +2536,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="17.25">
+    <row r="66" spans="1:3" ht="17.25" customHeight="1">
       <c r="A66" s="7" t="s">
         <v>55</v>
       </c>
@@ -2539,7 +2547,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="17.25">
+    <row r="67" spans="1:3" ht="17.25" customHeight="1">
       <c r="A67" s="7" t="s">
         <v>55</v>
       </c>
@@ -2550,7 +2558,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="17.25">
+    <row r="68" spans="1:3" ht="17.25" customHeight="1">
       <c r="A68" s="7" t="s">
         <v>55</v>
       </c>
@@ -2561,7 +2569,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="17.25">
+    <row r="69" spans="1:3" ht="17.25" customHeight="1">
       <c r="A69" s="7" t="s">
         <v>55</v>
       </c>
@@ -2572,7 +2580,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="17.25">
+    <row r="70" spans="1:3" ht="17.25" customHeight="1">
       <c r="A70" s="7" t="s">
         <v>55</v>
       </c>
@@ -2583,7 +2591,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="17.25">
+    <row r="71" spans="1:3" ht="17.25" customHeight="1">
       <c r="A71" s="7" t="s">
         <v>55</v>
       </c>
@@ -2594,7 +2602,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="17.25">
+    <row r="72" spans="1:3" ht="17.25" customHeight="1">
       <c r="A72" s="7" t="s">
         <v>55</v>
       </c>
@@ -2605,7 +2613,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="17.25">
+    <row r="73" spans="1:3" ht="17.25" customHeight="1">
       <c r="A73" s="7" t="s">
         <v>55</v>
       </c>
@@ -2616,7 +2624,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="17.25">
+    <row r="74" spans="1:3" ht="17.25" customHeight="1">
       <c r="A74" s="7" t="s">
         <v>55</v>
       </c>
@@ -2627,7 +2635,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="17.25">
+    <row r="75" spans="1:3" ht="17.25" customHeight="1">
       <c r="A75" s="7" t="s">
         <v>55</v>
       </c>
@@ -2638,7 +2646,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="17.25">
+    <row r="76" spans="1:3" ht="17.25" customHeight="1">
       <c r="A76" s="7" t="s">
         <v>55</v>
       </c>
@@ -2649,7 +2657,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="17.25">
+    <row r="77" spans="1:3" ht="17.25" customHeight="1">
       <c r="A77" s="7" t="s">
         <v>55</v>
       </c>
@@ -2660,7 +2668,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="17.25">
+    <row r="78" spans="1:3" ht="17.25" customHeight="1">
       <c r="A78" s="7" t="s">
         <v>55</v>
       </c>
@@ -2671,7 +2679,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="17.25">
+    <row r="79" spans="1:3" ht="17.25" customHeight="1">
       <c r="A79" s="7" t="s">
         <v>55</v>
       </c>
@@ -2682,7 +2690,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="17.25">
+    <row r="80" spans="1:3" ht="17.25" customHeight="1">
       <c r="A80" s="7" t="s">
         <v>55</v>
       </c>
@@ -2693,7 +2701,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="17.25">
+    <row r="81" spans="1:3" ht="17.25" customHeight="1">
       <c r="A81" s="7" t="s">
         <v>55</v>
       </c>
@@ -2704,7 +2712,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="17.25">
+    <row r="82" spans="1:3" ht="17.25" customHeight="1">
       <c r="A82" s="7" t="s">
         <v>55</v>
       </c>
@@ -2715,7 +2723,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="17.25">
+    <row r="83" spans="1:3" ht="17.25" customHeight="1">
       <c r="A83" s="7" t="s">
         <v>55</v>
       </c>
@@ -2726,7 +2734,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="17.25">
+    <row r="84" spans="1:3" ht="17.25" customHeight="1">
       <c r="A84" s="7" t="s">
         <v>55</v>
       </c>
@@ -2737,7 +2745,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="17.25">
+    <row r="85" spans="1:3" ht="17.25" customHeight="1">
       <c r="A85" s="7" t="s">
         <v>55</v>
       </c>
@@ -2748,7 +2756,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="17.25">
+    <row r="86" spans="1:3" ht="17.25" customHeight="1">
       <c r="A86" s="7" t="s">
         <v>55</v>
       </c>
@@ -2759,7 +2767,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="17.25">
+    <row r="87" spans="1:3" ht="17.25" customHeight="1">
       <c r="A87" s="7" t="s">
         <v>55</v>
       </c>
@@ -2770,7 +2778,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="17.25">
+    <row r="88" spans="1:3" ht="17.25" customHeight="1">
       <c r="A88" s="7" t="s">
         <v>55</v>
       </c>
@@ -2781,7 +2789,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="17.25">
+    <row r="89" spans="1:3" ht="17.25" customHeight="1">
       <c r="A89" s="7" t="s">
         <v>55</v>
       </c>
@@ -2792,7 +2800,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="17.25">
+    <row r="90" spans="1:3" ht="17.25" customHeight="1">
       <c r="A90" s="7" t="s">
         <v>55</v>
       </c>
@@ -2803,7 +2811,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="17.25">
+    <row r="91" spans="1:3" ht="17.25" customHeight="1">
       <c r="A91" s="7" t="s">
         <v>55</v>
       </c>
@@ -2814,7 +2822,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="17.25">
+    <row r="92" spans="1:3" ht="17.25" customHeight="1">
       <c r="A92" s="7" t="s">
         <v>55</v>
       </c>
@@ -2825,7 +2833,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="17.25">
+    <row r="93" spans="1:3" ht="17.25" customHeight="1">
       <c r="A93" s="7" t="s">
         <v>55</v>
       </c>
@@ -2836,7 +2844,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="17.25">
+    <row r="94" spans="1:3" ht="17.25" customHeight="1">
       <c r="A94" s="7" t="s">
         <v>55</v>
       </c>
@@ -2847,7 +2855,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="17.25">
+    <row r="95" spans="1:3" ht="17.25" customHeight="1">
       <c r="A95" s="7" t="s">
         <v>55</v>
       </c>
@@ -2858,7 +2866,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="17.25">
+    <row r="96" spans="1:3" ht="17.25" customHeight="1">
       <c r="A96" s="7" t="s">
         <v>55</v>
       </c>
@@ -2869,7 +2877,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="17.25">
+    <row r="97" spans="1:3" ht="17.25" customHeight="1">
       <c r="A97" s="7" t="s">
         <v>55</v>
       </c>
@@ -2880,7 +2888,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="17.25">
+    <row r="98" spans="1:3" ht="17.25" customHeight="1">
       <c r="A98" s="7" t="s">
         <v>55</v>
       </c>
@@ -2891,17 +2899,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="17.25">
+    <row r="99" spans="1:3" ht="17.25" customHeight="1">
       <c r="A99" s="1"/>
       <c r="B99" s="4"/>
       <c r="C99" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="17.25">
+    <row r="100" spans="1:3" ht="17.25" customHeight="1">
       <c r="A100" s="7"/>
       <c r="B100" s="9"/>
       <c r="C100" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="17.25">
+    <row r="101" spans="1:3" ht="17.25" customHeight="1">
       <c r="A101" s="7" t="s">
         <v>100</v>
       </c>
@@ -2912,7 +2920,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="17.25">
+    <row r="102" spans="1:3" ht="17.25" customHeight="1">
       <c r="A102" s="7" t="s">
         <v>100</v>
       </c>
@@ -2923,7 +2931,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="17.25">
+    <row r="103" spans="1:3" ht="17.25" customHeight="1">
       <c r="A103" s="7" t="s">
         <v>100</v>
       </c>
@@ -2934,7 +2942,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="17.25">
+    <row r="104" spans="1:3" ht="17.25" customHeight="1">
       <c r="A104" s="7" t="s">
         <v>100</v>
       </c>
@@ -2945,7 +2953,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="24">
+    <row r="105" spans="1:3" ht="24" customHeight="1">
       <c r="A105" s="7" t="s">
         <v>100</v>
       </c>
@@ -2956,7 +2964,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="24">
+    <row r="106" spans="1:3" ht="24" customHeight="1">
       <c r="A106" s="7" t="s">
         <v>100</v>
       </c>
@@ -2967,7 +2975,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="24">
+    <row r="107" spans="1:3" ht="24" customHeight="1">
       <c r="A107" s="7" t="s">
         <v>100</v>
       </c>
@@ -2978,7 +2986,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="24">
+    <row r="108" spans="1:3" ht="24" customHeight="1">
       <c r="A108" s="7" t="s">
         <v>100</v>
       </c>
@@ -2989,7 +2997,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="24">
+    <row r="109" spans="1:3" ht="24" customHeight="1">
       <c r="A109" s="7" t="s">
         <v>100</v>
       </c>
@@ -3000,7 +3008,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="24">
+    <row r="110" spans="1:3" ht="24" customHeight="1">
       <c r="A110" s="7" t="s">
         <v>100</v>
       </c>
@@ -3011,7 +3019,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="24">
+    <row r="111" spans="1:3" ht="24" customHeight="1">
       <c r="A111" s="7" t="s">
         <v>100</v>
       </c>
@@ -3022,7 +3030,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="24">
+    <row r="112" spans="1:3" ht="24" customHeight="1">
       <c r="A112" s="7" t="s">
         <v>100</v>
       </c>
@@ -3033,7 +3041,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="24">
+    <row r="113" spans="1:3" ht="24" customHeight="1">
       <c r="A113" s="7" t="s">
         <v>100</v>
       </c>
@@ -3044,7 +3052,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="24">
+    <row r="114" spans="1:3" ht="24" customHeight="1">
       <c r="A114" s="7" t="s">
         <v>100</v>
       </c>
@@ -3055,7 +3063,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="24">
+    <row r="115" spans="1:3" ht="24" customHeight="1">
       <c r="A115" s="7" t="s">
         <v>100</v>
       </c>
@@ -3066,7 +3074,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="24">
+    <row r="116" spans="1:3" ht="24" customHeight="1">
       <c r="A116" s="7" t="s">
         <v>100</v>
       </c>
@@ -3077,7 +3085,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="24">
+    <row r="117" spans="1:3" ht="24" customHeight="1">
       <c r="A117" s="7" t="s">
         <v>100</v>
       </c>
@@ -3088,7 +3096,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="24">
+    <row r="118" spans="1:3" ht="24" customHeight="1">
       <c r="A118" s="7" t="s">
         <v>100</v>
       </c>
@@ -3099,7 +3107,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="24">
+    <row r="119" spans="1:3" ht="24" customHeight="1">
       <c r="A119" s="7" t="s">
         <v>100</v>
       </c>
@@ -3110,7 +3118,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="24">
+    <row r="120" spans="1:3" ht="24" customHeight="1">
       <c r="A120" s="7" t="s">
         <v>100</v>
       </c>
@@ -3121,7 +3129,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="24">
+    <row r="121" spans="1:3" ht="24" customHeight="1">
       <c r="A121" s="7" t="s">
         <v>100</v>
       </c>
@@ -3132,7 +3140,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="17.25">
+    <row r="122" spans="1:3" ht="17.25" customHeight="1">
       <c r="A122" s="7" t="s">
         <v>100</v>
       </c>
@@ -3143,7 +3151,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="17.25">
+    <row r="123" spans="1:3" ht="17.25" customHeight="1">
       <c r="A123" s="7" t="s">
         <v>100</v>
       </c>
@@ -3154,7 +3162,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="17.25">
+    <row r="124" spans="1:3" ht="17.25" customHeight="1">
       <c r="A124" s="7" t="s">
         <v>100</v>
       </c>
@@ -3165,7 +3173,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="17.25">
+    <row r="125" spans="1:3" ht="17.25" customHeight="1">
       <c r="A125" s="7" t="s">
         <v>100</v>
       </c>
@@ -3176,7 +3184,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="17.25">
+    <row r="126" spans="1:3" ht="17.25" customHeight="1">
       <c r="A126" s="7" t="s">
         <v>100</v>
       </c>
@@ -3187,7 +3195,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="17.25">
+    <row r="127" spans="1:3" ht="17.25" customHeight="1">
       <c r="A127" s="7" t="s">
         <v>100</v>
       </c>
@@ -3198,7 +3206,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="17.25">
+    <row r="128" spans="1:3" ht="17.25" customHeight="1">
       <c r="A128" s="7" t="s">
         <v>100</v>
       </c>
@@ -3209,7 +3217,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="17.25">
+    <row r="129" spans="1:3" ht="17.25" customHeight="1">
       <c r="A129" s="7" t="s">
         <v>100</v>
       </c>
@@ -3220,7 +3228,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="17.25">
+    <row r="130" spans="1:3" ht="17.25" customHeight="1">
       <c r="A130" s="7" t="s">
         <v>100</v>
       </c>
@@ -3231,7 +3239,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="17.25">
+    <row r="131" spans="1:3" ht="17.25" customHeight="1">
       <c r="A131" s="7" t="s">
         <v>100</v>
       </c>
@@ -3242,7 +3250,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="17.25">
+    <row r="132" spans="1:3" ht="17.25" customHeight="1">
       <c r="A132" s="7" t="s">
         <v>100</v>
       </c>
@@ -3253,7 +3261,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="17.25">
+    <row r="133" spans="1:3" ht="17.25" customHeight="1">
       <c r="A133" s="7" t="s">
         <v>100</v>
       </c>
@@ -3264,7 +3272,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="17.25">
+    <row r="134" spans="1:3" ht="17.25" customHeight="1">
       <c r="A134" s="7" t="s">
         <v>100</v>
       </c>
@@ -3275,7 +3283,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="17.25">
+    <row r="135" spans="1:3" ht="17.25" customHeight="1">
       <c r="A135" s="7" t="s">
         <v>100</v>
       </c>
@@ -3286,7 +3294,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="17.25">
+    <row r="136" spans="1:3" ht="17.25" customHeight="1">
       <c r="A136" s="7" t="s">
         <v>100</v>
       </c>
@@ -3297,17 +3305,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="17.25">
+    <row r="137" spans="1:3" ht="17.25" customHeight="1">
       <c r="A137" s="1"/>
       <c r="B137" s="4"/>
       <c r="C137" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="17.25">
+    <row r="138" spans="1:3" ht="17.25" customHeight="1">
       <c r="A138" s="1"/>
       <c r="B138" s="9"/>
       <c r="C138" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="17.25">
+    <row r="139" spans="1:3" ht="17.25" customHeight="1">
       <c r="A139" s="7" t="s">
         <v>137</v>
       </c>
@@ -3318,7 +3326,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="17.25">
+    <row r="140" spans="1:3" ht="17.25" customHeight="1">
       <c r="A140" s="7" t="s">
         <v>137</v>
       </c>
@@ -3329,7 +3337,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="17.25">
+    <row r="141" spans="1:3" ht="17.25" customHeight="1">
       <c r="A141" s="7" t="s">
         <v>137</v>
       </c>
@@ -3340,7 +3348,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="17.25">
+    <row r="142" spans="1:3" ht="17.25" customHeight="1">
       <c r="A142" s="7" t="s">
         <v>137</v>
       </c>
@@ -3351,7 +3359,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="17.25">
+    <row r="143" spans="1:3" ht="17.25" customHeight="1">
       <c r="A143" s="7" t="s">
         <v>137</v>
       </c>
@@ -3362,7 +3370,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="17.25">
+    <row r="144" spans="1:3" ht="17.25" customHeight="1">
       <c r="A144" s="7" t="s">
         <v>137</v>
       </c>
@@ -3373,7 +3381,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="17.25">
+    <row r="145" spans="1:3" ht="17.25" customHeight="1">
       <c r="A145" s="7" t="s">
         <v>137</v>
       </c>
@@ -3384,7 +3392,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="17.25">
+    <row r="146" spans="1:3" ht="17.25" customHeight="1">
       <c r="A146" s="7" t="s">
         <v>137</v>
       </c>
@@ -3395,7 +3403,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="17.25">
+    <row r="147" spans="1:3" ht="17.25" customHeight="1">
       <c r="A147" s="7" t="s">
         <v>137</v>
       </c>
@@ -3406,7 +3414,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="17.25">
+    <row r="148" spans="1:3" ht="17.25" customHeight="1">
       <c r="A148" s="7" t="s">
         <v>137</v>
       </c>
@@ -3417,7 +3425,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="17.25">
+    <row r="149" spans="1:3" ht="17.25" customHeight="1">
       <c r="A149" s="7" t="s">
         <v>137</v>
       </c>
@@ -3428,7 +3436,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="17.25">
+    <row r="150" spans="1:3" ht="17.25" customHeight="1">
       <c r="A150" s="7" t="s">
         <v>137</v>
       </c>
@@ -3439,7 +3447,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="17.25">
+    <row r="151" spans="1:3" ht="17.25" customHeight="1">
       <c r="A151" s="7" t="s">
         <v>137</v>
       </c>
@@ -3450,7 +3458,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="17.25">
+    <row r="152" spans="1:3" ht="17.25" customHeight="1">
       <c r="A152" s="7" t="s">
         <v>137</v>
       </c>
@@ -3461,7 +3469,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="17.25">
+    <row r="153" spans="1:3" ht="17.25" customHeight="1">
       <c r="A153" s="7" t="s">
         <v>137</v>
       </c>
@@ -3472,7 +3480,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="17.25">
+    <row r="154" spans="1:3" ht="17.25" customHeight="1">
       <c r="A154" s="7" t="s">
         <v>137</v>
       </c>
@@ -3483,7 +3491,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="17.25">
+    <row r="155" spans="1:3" ht="17.25" customHeight="1">
       <c r="A155" s="7" t="s">
         <v>137</v>
       </c>
@@ -3494,7 +3502,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="17.25">
+    <row r="156" spans="1:3" ht="17.25" customHeight="1">
       <c r="A156" s="7" t="s">
         <v>137</v>
       </c>
@@ -3505,7 +3513,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="17.25">
+    <row r="157" spans="1:3" ht="17.25" customHeight="1">
       <c r="A157" s="7" t="s">
         <v>137</v>
       </c>
@@ -3516,7 +3524,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="17.25">
+    <row r="158" spans="1:3" ht="17.25" customHeight="1">
       <c r="A158" s="7" t="s">
         <v>137</v>
       </c>
@@ -3527,7 +3535,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="17.25">
+    <row r="159" spans="1:3" ht="17.25" customHeight="1">
       <c r="A159" s="7" t="s">
         <v>137</v>
       </c>
@@ -3538,7 +3546,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="17.25">
+    <row r="160" spans="1:3" ht="17.25" customHeight="1">
       <c r="A160" s="7" t="s">
         <v>137</v>
       </c>
@@ -3549,7 +3557,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="17.25">
+    <row r="161" spans="1:3" ht="17.25" customHeight="1">
       <c r="A161" s="7" t="s">
         <v>137</v>
       </c>
@@ -3560,7 +3568,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="17.25">
+    <row r="162" spans="1:3" ht="17.25" customHeight="1">
       <c r="A162" s="7" t="s">
         <v>137</v>
       </c>
@@ -3571,7 +3579,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="17.25">
+    <row r="163" spans="1:3" ht="17.25" customHeight="1">
       <c r="A163" s="7" t="s">
         <v>137</v>
       </c>
@@ -3582,7 +3590,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="17.25">
+    <row r="164" spans="1:3" ht="17.25" customHeight="1">
       <c r="A164" s="7" t="s">
         <v>137</v>
       </c>
@@ -3593,7 +3601,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="17.25">
+    <row r="165" spans="1:3" ht="17.25" customHeight="1">
       <c r="A165" s="7" t="s">
         <v>137</v>
       </c>
@@ -3604,7 +3612,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="17.25">
+    <row r="166" spans="1:3" ht="17.25" customHeight="1">
       <c r="A166" s="7" t="s">
         <v>137</v>
       </c>
@@ -3615,7 +3623,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="17.25">
+    <row r="167" spans="1:3" ht="17.25" customHeight="1">
       <c r="A167" s="7" t="s">
         <v>137</v>
       </c>
@@ -3626,7 +3634,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="17.25">
+    <row r="168" spans="1:3" ht="17.25" customHeight="1">
       <c r="A168" s="7" t="s">
         <v>137</v>
       </c>
@@ -3637,7 +3645,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="17.25">
+    <row r="169" spans="1:3" ht="17.25" customHeight="1">
       <c r="A169" s="7" t="s">
         <v>137</v>
       </c>
@@ -3648,7 +3656,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="17.25">
+    <row r="170" spans="1:3" ht="17.25" customHeight="1">
       <c r="A170" s="7" t="s">
         <v>137</v>
       </c>
@@ -3659,7 +3667,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="17.25">
+    <row r="171" spans="1:3" ht="17.25" customHeight="1">
       <c r="A171" s="7" t="s">
         <v>137</v>
       </c>
@@ -3670,7 +3678,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="17.25">
+    <row r="172" spans="1:3" ht="17.25" customHeight="1">
       <c r="A172" s="7" t="s">
         <v>137</v>
       </c>
@@ -3681,7 +3689,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="17.25">
+    <row r="173" spans="1:3" ht="17.25" customHeight="1">
       <c r="A173" s="7" t="s">
         <v>137</v>
       </c>
@@ -3692,7 +3700,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="17.25">
+    <row r="174" spans="1:3" ht="17.25" customHeight="1">
       <c r="A174" s="7" t="s">
         <v>137</v>
       </c>
@@ -3703,17 +3711,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="17.25">
+    <row r="175" spans="1:3" ht="17.25" customHeight="1">
       <c r="A175" s="1"/>
       <c r="B175" s="4"/>
       <c r="C175" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="17.25">
+    <row r="176" spans="1:3" ht="17.25" customHeight="1">
       <c r="A176" s="1"/>
       <c r="B176" s="9"/>
       <c r="C176" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="17.25">
+    <row r="177" spans="1:3" ht="17.25" customHeight="1">
       <c r="A177" s="7" t="s">
         <v>174</v>
       </c>
@@ -3724,7 +3732,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="17.25">
+    <row r="178" spans="1:3" ht="17.25" customHeight="1">
       <c r="A178" s="7" t="s">
         <v>174</v>
       </c>
@@ -3735,7 +3743,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="17.25">
+    <row r="179" spans="1:3" ht="17.25" customHeight="1">
       <c r="A179" s="7" t="s">
         <v>174</v>
       </c>
@@ -3746,7 +3754,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="17.25">
+    <row r="180" spans="1:3" ht="17.25" customHeight="1">
       <c r="A180" s="7" t="s">
         <v>174</v>
       </c>
@@ -3757,7 +3765,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="17.25">
+    <row r="181" spans="1:3" ht="17.25" customHeight="1">
       <c r="A181" s="7" t="s">
         <v>174</v>
       </c>
@@ -3768,7 +3776,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="17.25">
+    <row r="182" spans="1:3" ht="17.25" customHeight="1">
       <c r="A182" s="7" t="s">
         <v>174</v>
       </c>
@@ -3779,7 +3787,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="17.25">
+    <row r="183" spans="1:3" ht="17.25" customHeight="1">
       <c r="A183" s="7" t="s">
         <v>174</v>
       </c>
@@ -3790,7 +3798,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="17.25">
+    <row r="184" spans="1:3" ht="17.25" customHeight="1">
       <c r="A184" s="7" t="s">
         <v>174</v>
       </c>
@@ -3801,7 +3809,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="17.25">
+    <row r="185" spans="1:3" ht="17.25" customHeight="1">
       <c r="A185" s="7" t="s">
         <v>174</v>
       </c>
@@ -3812,7 +3820,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="17.25">
+    <row r="186" spans="1:3" ht="17.25" customHeight="1">
       <c r="A186" s="7" t="s">
         <v>174</v>
       </c>
@@ -3823,7 +3831,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="17.25">
+    <row r="187" spans="1:3" ht="17.25" customHeight="1">
       <c r="A187" s="7" t="s">
         <v>174</v>
       </c>
@@ -3834,7 +3842,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="17.25">
+    <row r="188" spans="1:3" ht="17.25" customHeight="1">
       <c r="A188" s="7" t="s">
         <v>174</v>
       </c>
@@ -3845,7 +3853,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="17.25">
+    <row r="189" spans="1:3" ht="17.25" customHeight="1">
       <c r="A189" s="7" t="s">
         <v>174</v>
       </c>
@@ -3856,7 +3864,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="17.25">
+    <row r="190" spans="1:3" ht="17.25" customHeight="1">
       <c r="A190" s="7" t="s">
         <v>174</v>
       </c>
@@ -3867,7 +3875,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="17.25">
+    <row r="191" spans="1:3" ht="17.25" customHeight="1">
       <c r="A191" s="7" t="s">
         <v>174</v>
       </c>
@@ -3878,7 +3886,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="17.25">
+    <row r="192" spans="1:3" ht="17.25" customHeight="1">
       <c r="A192" s="7" t="s">
         <v>174</v>
       </c>
@@ -3889,7 +3897,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="17.25">
+    <row r="193" spans="1:3" ht="17.25" customHeight="1">
       <c r="A193" s="7" t="s">
         <v>174</v>
       </c>
@@ -3900,7 +3908,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="17.25">
+    <row r="194" spans="1:3" ht="17.25" customHeight="1">
       <c r="A194" s="7" t="s">
         <v>174</v>
       </c>
@@ -3911,7 +3919,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="17.25">
+    <row r="195" spans="1:3" ht="17.25" customHeight="1">
       <c r="A195" s="7" t="s">
         <v>174</v>
       </c>
@@ -3922,7 +3930,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="17.25">
+    <row r="196" spans="1:3" ht="17.25" customHeight="1">
       <c r="A196" s="7" t="s">
         <v>174</v>
       </c>
@@ -3933,7 +3941,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="17.25">
+    <row r="197" spans="1:3" ht="17.25" customHeight="1">
       <c r="A197" s="7" t="s">
         <v>174</v>
       </c>
@@ -3944,7 +3952,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="17.25">
+    <row r="198" spans="1:3" ht="17.25" customHeight="1">
       <c r="A198" s="7" t="s">
         <v>174</v>
       </c>
@@ -3955,7 +3963,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="17.25">
+    <row r="199" spans="1:3" ht="17.25" customHeight="1">
       <c r="A199" s="7" t="s">
         <v>174</v>
       </c>
@@ -3966,7 +3974,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="17.25">
+    <row r="200" spans="1:3" ht="17.25" customHeight="1">
       <c r="A200" s="7" t="s">
         <v>174</v>
       </c>
@@ -3977,7 +3985,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="17.25">
+    <row r="201" spans="1:3" ht="17.25" customHeight="1">
       <c r="A201" s="7" t="s">
         <v>174</v>
       </c>
@@ -3988,7 +3996,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="17.25">
+    <row r="202" spans="1:3" ht="17.25" customHeight="1">
       <c r="A202" s="7" t="s">
         <v>174</v>
       </c>
@@ -3999,7 +4007,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="17.25">
+    <row r="203" spans="1:3" ht="17.25" customHeight="1">
       <c r="A203" s="7" t="s">
         <v>174</v>
       </c>
@@ -4010,7 +4018,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="17.25">
+    <row r="204" spans="1:3" ht="17.25" customHeight="1">
       <c r="A204" s="7" t="s">
         <v>174</v>
       </c>
@@ -4021,7 +4029,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="17.25">
+    <row r="205" spans="1:3" ht="17.25" customHeight="1">
       <c r="A205" s="7" t="s">
         <v>174</v>
       </c>
@@ -4032,7 +4040,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="17.25">
+    <row r="206" spans="1:3" ht="17.25" customHeight="1">
       <c r="A206" s="7" t="s">
         <v>174</v>
       </c>
@@ -4043,7 +4051,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="17.25">
+    <row r="207" spans="1:3" ht="17.25" customHeight="1">
       <c r="A207" s="7" t="s">
         <v>174</v>
       </c>
@@ -4054,7 +4062,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="17.25">
+    <row r="208" spans="1:3" ht="17.25" customHeight="1">
       <c r="A208" s="7" t="s">
         <v>174</v>
       </c>
@@ -4065,7 +4073,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="209" customHeight="1" ht="17.25">
+    <row r="209" spans="1:3" ht="17.25" customHeight="1">
       <c r="A209" s="7" t="s">
         <v>174</v>
       </c>
@@ -4076,7 +4084,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="210" customHeight="1" ht="17.25">
+    <row r="210" spans="1:3" ht="17.25" customHeight="1">
       <c r="A210" s="7" t="s">
         <v>174</v>
       </c>
@@ -4087,7 +4095,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="211" customHeight="1" ht="17.25">
+    <row r="211" spans="1:3" ht="17.25" customHeight="1">
       <c r="A211" s="7" t="s">
         <v>174</v>
       </c>
@@ -4098,17 +4106,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="212" customHeight="1" ht="17.25">
+    <row r="212" spans="1:3" ht="17.25" customHeight="1">
       <c r="A212" s="7"/>
       <c r="B212" s="9"/>
       <c r="C212" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="213" customHeight="1" ht="17.25">
+    <row r="213" spans="1:3" ht="17.25" customHeight="1">
       <c r="A213" s="7"/>
       <c r="B213" s="9"/>
       <c r="C213" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="214" customHeight="1" ht="17.25">
+    <row r="214" spans="1:3" ht="17.25" customHeight="1">
       <c r="A214" s="7" t="s">
         <v>210</v>
       </c>
@@ -4119,7 +4127,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="215" customHeight="1" ht="17.25">
+    <row r="215" spans="1:3" ht="17.25" customHeight="1">
       <c r="A215" s="7" t="s">
         <v>210</v>
       </c>
@@ -4130,7 +4138,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="216" customHeight="1" ht="17.25">
+    <row r="216" spans="1:3" ht="17.25" customHeight="1">
       <c r="A216" s="7" t="s">
         <v>210</v>
       </c>
@@ -4141,7 +4149,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="217" customHeight="1" ht="17.25">
+    <row r="217" spans="1:3" ht="17.25" customHeight="1">
       <c r="A217" s="7" t="s">
         <v>210</v>
       </c>
@@ -4152,7 +4160,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="17.25">
+    <row r="218" spans="1:3" ht="17.25" customHeight="1">
       <c r="A218" s="7" t="s">
         <v>210</v>
       </c>
@@ -4163,7 +4171,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="17.25">
+    <row r="219" spans="1:3" ht="17.25" customHeight="1">
       <c r="A219" s="7" t="s">
         <v>210</v>
       </c>
@@ -4174,7 +4182,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="220" customHeight="1" ht="17.25">
+    <row r="220" spans="1:3" ht="17.25" customHeight="1">
       <c r="A220" s="7" t="s">
         <v>210</v>
       </c>
@@ -4185,7 +4193,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="17.25">
+    <row r="221" spans="1:3" ht="17.25" customHeight="1">
       <c r="A221" s="7" t="s">
         <v>210</v>
       </c>
@@ -4196,7 +4204,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="17.25">
+    <row r="222" spans="1:3" ht="17.25" customHeight="1">
       <c r="A222" s="7" t="s">
         <v>210</v>
       </c>
@@ -4207,7 +4215,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="17.25">
+    <row r="223" spans="1:3" ht="17.25" customHeight="1">
       <c r="A223" s="7" t="s">
         <v>210</v>
       </c>
@@ -4218,7 +4226,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="17.25">
+    <row r="224" spans="1:3" ht="17.25" customHeight="1">
       <c r="A224" s="7" t="s">
         <v>210</v>
       </c>
@@ -4229,7 +4237,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="17.25">
+    <row r="225" spans="1:3" ht="17.25" customHeight="1">
       <c r="A225" s="7" t="s">
         <v>210</v>
       </c>
@@ -4240,7 +4248,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="17.25">
+    <row r="226" spans="1:3" ht="17.25" customHeight="1">
       <c r="A226" s="7" t="s">
         <v>210</v>
       </c>
@@ -4251,7 +4259,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="17.25">
+    <row r="227" spans="1:3" ht="17.25" customHeight="1">
       <c r="A227" s="7" t="s">
         <v>210</v>
       </c>
@@ -4262,7 +4270,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="17.25">
+    <row r="228" spans="1:3" ht="17.25" customHeight="1">
       <c r="A228" s="7" t="s">
         <v>210</v>
       </c>
@@ -4273,7 +4281,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="17.25">
+    <row r="229" spans="1:3" ht="17.25" customHeight="1">
       <c r="A229" s="7" t="s">
         <v>210</v>
       </c>
@@ -4284,7 +4292,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="230" customHeight="1" ht="17.25">
+    <row r="230" spans="1:3" ht="17.25" customHeight="1">
       <c r="A230" s="7" t="s">
         <v>210</v>
       </c>
@@ -4295,7 +4303,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="231" customHeight="1" ht="17.25">
+    <row r="231" spans="1:3" ht="17.25" customHeight="1">
       <c r="A231" s="7" t="s">
         <v>210</v>
       </c>
@@ -4306,7 +4314,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="232" customHeight="1" ht="17.25">
+    <row r="232" spans="1:3" ht="17.25" customHeight="1">
       <c r="A232" s="7" t="s">
         <v>210</v>
       </c>
@@ -4317,7 +4325,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="233" customHeight="1" ht="17.25">
+    <row r="233" spans="1:3" ht="17.25" customHeight="1">
       <c r="A233" s="7" t="s">
         <v>210</v>
       </c>
@@ -4328,7 +4336,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="234" customHeight="1" ht="17.25">
+    <row r="234" spans="1:3" ht="17.25" customHeight="1">
       <c r="A234" s="7" t="s">
         <v>210</v>
       </c>
@@ -4339,7 +4347,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="235" customHeight="1" ht="17.25">
+    <row r="235" spans="1:3" ht="17.25" customHeight="1">
       <c r="A235" s="7" t="s">
         <v>210</v>
       </c>
@@ -4350,17 +4358,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="236" customHeight="1" ht="17.25">
+    <row r="236" spans="1:3" ht="17.25" customHeight="1">
       <c r="A236" s="1"/>
       <c r="B236" s="9"/>
       <c r="C236" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="237" customHeight="1" ht="17.25">
+    <row r="237" spans="1:3" ht="17.25" customHeight="1">
       <c r="A237" s="1"/>
       <c r="B237" s="9"/>
       <c r="C237" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="238" customHeight="1" ht="17.25">
+    <row r="238" spans="1:3" ht="17.25" customHeight="1">
       <c r="A238" s="7" t="s">
         <v>233</v>
       </c>
@@ -4371,7 +4379,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="239" customHeight="1" ht="17.25">
+    <row r="239" spans="1:3" ht="17.25" customHeight="1">
       <c r="A239" s="7" t="s">
         <v>233</v>
       </c>
@@ -4382,7 +4390,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="240" customHeight="1" ht="17.25">
+    <row r="240" spans="1:3" ht="17.25" customHeight="1">
       <c r="A240" s="7" t="s">
         <v>233</v>
       </c>
@@ -4393,7 +4401,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="241" customHeight="1" ht="17.25">
+    <row r="241" spans="1:3" ht="17.25" customHeight="1">
       <c r="A241" s="7" t="s">
         <v>233</v>
       </c>
@@ -4404,7 +4412,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="242" customHeight="1" ht="17.25">
+    <row r="242" spans="1:3" ht="17.25" customHeight="1">
       <c r="A242" s="7" t="s">
         <v>233</v>
       </c>
@@ -4415,7 +4423,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="243" customHeight="1" ht="17.25">
+    <row r="243" spans="1:3" ht="17.25" customHeight="1">
       <c r="A243" s="7" t="s">
         <v>233</v>
       </c>
@@ -4426,7 +4434,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="244" customHeight="1" ht="17.25">
+    <row r="244" spans="1:3" ht="17.25" customHeight="1">
       <c r="A244" s="7" t="s">
         <v>233</v>
       </c>
@@ -4437,7 +4445,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="245" customHeight="1" ht="17.25">
+    <row r="245" spans="1:3" ht="17.25" customHeight="1">
       <c r="A245" s="7" t="s">
         <v>233</v>
       </c>
@@ -4448,7 +4456,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="17.25">
+    <row r="246" spans="1:3" ht="17.25" customHeight="1">
       <c r="A246" s="7" t="s">
         <v>233</v>
       </c>
@@ -4459,7 +4467,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="17.25">
+    <row r="247" spans="1:3" ht="17.25" customHeight="1">
       <c r="A247" s="7" t="s">
         <v>233</v>
       </c>
@@ -4470,7 +4478,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="248" customHeight="1" ht="17.25">
+    <row r="248" spans="1:3" ht="17.25" customHeight="1">
       <c r="A248" s="7" t="s">
         <v>233</v>
       </c>
@@ -4481,7 +4489,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="17.25">
+    <row r="249" spans="1:3" ht="17.25" customHeight="1">
       <c r="A249" s="7" t="s">
         <v>233</v>
       </c>
@@ -4492,7 +4500,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="17.25">
+    <row r="250" spans="1:3" ht="17.25" customHeight="1">
       <c r="A250" s="7" t="s">
         <v>233</v>
       </c>
@@ -4503,7 +4511,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="251" customHeight="1" ht="17.25">
+    <row r="251" spans="1:3" ht="17.25" customHeight="1">
       <c r="A251" s="7" t="s">
         <v>233</v>
       </c>
@@ -4514,7 +4522,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="252" customHeight="1" ht="17.25">
+    <row r="252" spans="1:3" ht="17.25" customHeight="1">
       <c r="A252" s="7" t="s">
         <v>233</v>
       </c>
@@ -4525,7 +4533,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="253" customHeight="1" ht="17.25">
+    <row r="253" spans="1:3" ht="17.25" customHeight="1">
       <c r="A253" s="7" t="s">
         <v>233</v>
       </c>
@@ -4536,7 +4544,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="17.25">
+    <row r="254" spans="1:3" ht="17.25" customHeight="1">
       <c r="A254" s="7" t="s">
         <v>233</v>
       </c>
@@ -4547,7 +4555,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="17.25">
+    <row r="255" spans="1:3" ht="17.25" customHeight="1">
       <c r="A255" s="7" t="s">
         <v>233</v>
       </c>
@@ -4558,7 +4566,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="17.25">
+    <row r="256" spans="1:3" ht="17.25" customHeight="1">
       <c r="A256" s="7" t="s">
         <v>233</v>
       </c>
@@ -4569,7 +4577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="257" customHeight="1" ht="17.25">
+    <row r="257" spans="1:3" ht="17.25" customHeight="1">
       <c r="A257" s="7" t="s">
         <v>233</v>
       </c>
@@ -4580,7 +4588,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="17.25">
+    <row r="258" spans="1:3" ht="17.25" customHeight="1">
       <c r="A258" s="7" t="s">
         <v>233</v>
       </c>
@@ -4591,7 +4599,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="259" customHeight="1" ht="17.25">
+    <row r="259" spans="1:3" ht="17.25" customHeight="1">
       <c r="A259" s="7" t="s">
         <v>233</v>
       </c>
@@ -4602,7 +4610,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="17.25">
+    <row r="260" spans="1:3" ht="17.25" customHeight="1">
       <c r="A260" s="7" t="s">
         <v>233</v>
       </c>
@@ -4613,7 +4621,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="17.25">
+    <row r="261" spans="1:3" ht="17.25" customHeight="1">
       <c r="A261" s="7" t="s">
         <v>233</v>
       </c>
@@ -4624,7 +4632,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="17.25">
+    <row r="262" spans="1:3" ht="17.25" customHeight="1">
       <c r="A262" s="7" t="s">
         <v>233</v>
       </c>
@@ -4635,7 +4643,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="17.25">
+    <row r="263" spans="1:3" ht="17.25" customHeight="1">
       <c r="A263" s="7" t="s">
         <v>233</v>
       </c>
@@ -4646,7 +4654,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="17.25">
+    <row r="264" spans="1:3" ht="17.25" customHeight="1">
       <c r="A264" s="7" t="s">
         <v>233</v>
       </c>
@@ -4657,7 +4665,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="17.25">
+    <row r="265" spans="1:3" ht="17.25" customHeight="1">
       <c r="A265" s="7" t="s">
         <v>233</v>
       </c>
@@ -4668,7 +4676,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="17.25">
+    <row r="266" spans="1:3" ht="17.25" customHeight="1">
       <c r="A266" s="7" t="s">
         <v>233</v>
       </c>
@@ -4679,7 +4687,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="17.25">
+    <row r="267" spans="1:3" ht="17.25" customHeight="1">
       <c r="A267" s="7" t="s">
         <v>233</v>
       </c>
@@ -4690,7 +4698,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="17.25">
+    <row r="268" spans="1:3" ht="17.25" customHeight="1">
       <c r="A268" s="7" t="s">
         <v>233</v>
       </c>
@@ -4701,7 +4709,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="17.25">
+    <row r="269" spans="1:3" ht="17.25" customHeight="1">
       <c r="A269" s="7" t="s">
         <v>233</v>
       </c>
@@ -4712,7 +4720,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="270" customHeight="1" ht="17.25">
+    <row r="270" spans="1:3" ht="17.25" customHeight="1">
       <c r="A270" s="7" t="s">
         <v>233</v>
       </c>
@@ -4723,7 +4731,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="17.25">
+    <row r="271" spans="1:3" ht="17.25" customHeight="1">
       <c r="A271" s="7" t="s">
         <v>233</v>
       </c>
@@ -4734,7 +4742,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="17.25">
+    <row r="272" spans="1:3" ht="17.25" customHeight="1">
       <c r="A272" s="7" t="s">
         <v>233</v>
       </c>
@@ -4745,17 +4753,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="273" customHeight="1" ht="17.25">
+    <row r="273" spans="1:3" ht="17.25" customHeight="1">
       <c r="A273" s="1"/>
       <c r="B273" s="9"/>
       <c r="C273" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="17.25">
+    <row r="274" spans="1:3" ht="17.25" customHeight="1">
       <c r="A274" s="1"/>
       <c r="B274" s="9"/>
       <c r="C274" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="275" customHeight="1" ht="17.25">
+    <row r="275" spans="1:3" ht="17.25" customHeight="1">
       <c r="A275" s="7" t="s">
         <v>268</v>
       </c>
@@ -4766,7 +4774,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="17.25">
+    <row r="276" spans="1:3" ht="17.25" customHeight="1">
       <c r="A276" s="7" t="s">
         <v>268</v>
       </c>
@@ -4777,7 +4785,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="277" customHeight="1" ht="17.25">
+    <row r="277" spans="1:3" ht="17.25" customHeight="1">
       <c r="A277" s="7" t="s">
         <v>268</v>
       </c>
@@ -4788,7 +4796,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="17.25">
+    <row r="278" spans="1:3" ht="17.25" customHeight="1">
       <c r="A278" s="7" t="s">
         <v>268</v>
       </c>
@@ -4799,7 +4807,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="279" customHeight="1" ht="17.25">
+    <row r="279" spans="1:3" ht="17.25" customHeight="1">
       <c r="A279" s="7" t="s">
         <v>268</v>
       </c>
@@ -4810,7 +4818,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="280" customHeight="1" ht="17.25">
+    <row r="280" spans="1:3" ht="17.25" customHeight="1">
       <c r="A280" s="7" t="s">
         <v>268</v>
       </c>
@@ -4821,7 +4829,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="281" customHeight="1" ht="17.25">
+    <row r="281" spans="1:3" ht="17.25" customHeight="1">
       <c r="A281" s="7" t="s">
         <v>268</v>
       </c>
@@ -4832,7 +4840,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="282" customHeight="1" ht="17.25">
+    <row r="282" spans="1:3" ht="17.25" customHeight="1">
       <c r="A282" s="7" t="s">
         <v>268</v>
       </c>
@@ -4843,7 +4851,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="283" customHeight="1" ht="17.25">
+    <row r="283" spans="1:3" ht="17.25" customHeight="1">
       <c r="A283" s="7" t="s">
         <v>268</v>
       </c>
@@ -4854,7 +4862,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="17.25">
+    <row r="284" spans="1:3" ht="17.25" customHeight="1">
       <c r="A284" s="7" t="s">
         <v>268</v>
       </c>
@@ -4865,7 +4873,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="285" customHeight="1" ht="17.25">
+    <row r="285" spans="1:3" ht="17.25" customHeight="1">
       <c r="A285" s="7" t="s">
         <v>268</v>
       </c>
@@ -4876,7 +4884,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="286" customHeight="1" ht="17.25">
+    <row r="286" spans="1:3" ht="17.25" customHeight="1">
       <c r="A286" s="7" t="s">
         <v>268</v>
       </c>
@@ -4887,7 +4895,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="287" customHeight="1" ht="17.25">
+    <row r="287" spans="1:3" ht="17.25" customHeight="1">
       <c r="A287" s="7" t="s">
         <v>268</v>
       </c>
@@ -4898,7 +4906,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="288" customHeight="1" ht="17.25">
+    <row r="288" spans="1:3" ht="17.25" customHeight="1">
       <c r="A288" s="7" t="s">
         <v>268</v>
       </c>
@@ -4909,7 +4917,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="289" customHeight="1" ht="17.25">
+    <row r="289" spans="1:3" ht="17.25" customHeight="1">
       <c r="A289" s="7" t="s">
         <v>268</v>
       </c>
@@ -4920,7 +4928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="290" customHeight="1" ht="17.25">
+    <row r="290" spans="1:3" ht="17.25" customHeight="1">
       <c r="A290" s="7" t="s">
         <v>268</v>
       </c>
@@ -4931,7 +4939,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="291" customHeight="1" ht="17.25">
+    <row r="291" spans="1:3" ht="17.25" customHeight="1">
       <c r="A291" s="7" t="s">
         <v>268</v>
       </c>
@@ -4942,7 +4950,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="292" customHeight="1" ht="17.25">
+    <row r="292" spans="1:3" ht="17.25" customHeight="1">
       <c r="A292" s="7" t="s">
         <v>268</v>
       </c>
@@ -4953,7 +4961,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="293" customHeight="1" ht="17.25">
+    <row r="293" spans="1:3" ht="17.25" customHeight="1">
       <c r="A293" s="7" t="s">
         <v>268</v>
       </c>
@@ -4964,17 +4972,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="294" customHeight="1" ht="17.25">
+    <row r="294" spans="1:3" ht="17.25" customHeight="1">
       <c r="A294" s="1"/>
       <c r="B294" s="9"/>
       <c r="C294" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="295" customHeight="1" ht="17.25">
+    <row r="295" spans="1:3" ht="17.25" customHeight="1">
       <c r="A295" s="1"/>
       <c r="B295" s="9"/>
       <c r="C295" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="296" customHeight="1" ht="17.25">
+    <row r="296" spans="1:3" ht="17.25" customHeight="1">
       <c r="A296" s="7" t="s">
         <v>288</v>
       </c>
@@ -4985,7 +4993,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="297" customHeight="1" ht="17.25">
+    <row r="297" spans="1:3" ht="17.25" customHeight="1">
       <c r="A297" s="7" t="s">
         <v>288</v>
       </c>
@@ -4996,7 +5004,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="298" customHeight="1" ht="17.25">
+    <row r="298" spans="1:3" ht="17.25" customHeight="1">
       <c r="A298" s="7" t="s">
         <v>288</v>
       </c>
@@ -5007,7 +5015,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="299" customHeight="1" ht="17.25">
+    <row r="299" spans="1:3" ht="17.25" customHeight="1">
       <c r="A299" s="7" t="s">
         <v>288</v>
       </c>
@@ -5018,7 +5026,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="300" customHeight="1" ht="17.25">
+    <row r="300" spans="1:3" ht="17.25" customHeight="1">
       <c r="A300" s="7" t="s">
         <v>288</v>
       </c>
@@ -5029,7 +5037,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="301" customHeight="1" ht="17.25">
+    <row r="301" spans="1:3" ht="17.25" customHeight="1">
       <c r="A301" s="7" t="s">
         <v>288</v>
       </c>
@@ -5040,7 +5048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="302" customHeight="1" ht="17.25">
+    <row r="302" spans="1:3" ht="17.25" customHeight="1">
       <c r="A302" s="7" t="s">
         <v>288</v>
       </c>
@@ -5051,7 +5059,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="303" customHeight="1" ht="17.25">
+    <row r="303" spans="1:3" ht="17.25" customHeight="1">
       <c r="A303" s="7" t="s">
         <v>288</v>
       </c>
@@ -5062,7 +5070,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="304" customHeight="1" ht="17.25">
+    <row r="304" spans="1:3" ht="17.25" customHeight="1">
       <c r="A304" s="7" t="s">
         <v>288</v>
       </c>
@@ -5073,7 +5081,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="305" customHeight="1" ht="17.25">
+    <row r="305" spans="1:3" ht="17.25" customHeight="1">
       <c r="A305" s="7" t="s">
         <v>288</v>
       </c>
@@ -5084,7 +5092,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="306" customHeight="1" ht="17.25">
+    <row r="306" spans="1:3" ht="17.25" customHeight="1">
       <c r="A306" s="7" t="s">
         <v>288</v>
       </c>
@@ -5095,7 +5103,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="307" customHeight="1" ht="17.25">
+    <row r="307" spans="1:3" ht="17.25" customHeight="1">
       <c r="A307" s="7" t="s">
         <v>288</v>
       </c>
@@ -5106,7 +5114,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="308" customHeight="1" ht="17.25">
+    <row r="308" spans="1:3" ht="17.25" customHeight="1">
       <c r="A308" s="7" t="s">
         <v>288</v>
       </c>
@@ -5117,7 +5125,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="309" customHeight="1" ht="17.25">
+    <row r="309" spans="1:3" ht="17.25" customHeight="1">
       <c r="A309" s="7" t="s">
         <v>288</v>
       </c>
@@ -5128,7 +5136,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="310" customHeight="1" ht="17.25">
+    <row r="310" spans="1:3" ht="17.25" customHeight="1">
       <c r="A310" s="7" t="s">
         <v>288</v>
       </c>
@@ -5139,7 +5147,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="311" customHeight="1" ht="17.25">
+    <row r="311" spans="1:3" ht="17.25" customHeight="1">
       <c r="A311" s="7" t="s">
         <v>288</v>
       </c>
@@ -5150,7 +5158,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="312" customHeight="1" ht="17.25">
+    <row r="312" spans="1:3" ht="17.25" customHeight="1">
       <c r="A312" s="7" t="s">
         <v>288</v>
       </c>
@@ -5161,7 +5169,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="313" customHeight="1" ht="17.25">
+    <row r="313" spans="1:3" ht="17.25" customHeight="1">
       <c r="A313" s="7" t="s">
         <v>288</v>
       </c>
@@ -5172,7 +5180,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="314" customHeight="1" ht="17.25">
+    <row r="314" spans="1:3" ht="17.25" customHeight="1">
       <c r="A314" s="7" t="s">
         <v>288</v>
       </c>
@@ -5183,7 +5191,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="315" customHeight="1" ht="17.25">
+    <row r="315" spans="1:3" ht="17.25" customHeight="1">
       <c r="A315" s="7" t="s">
         <v>288</v>
       </c>
@@ -5194,7 +5202,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="316" customHeight="1" ht="17.25">
+    <row r="316" spans="1:3" ht="17.25" customHeight="1">
       <c r="A316" s="7" t="s">
         <v>288</v>
       </c>
@@ -5205,7 +5213,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="317" customHeight="1" ht="17.25">
+    <row r="317" spans="1:3" ht="17.25" customHeight="1">
       <c r="A317" s="7" t="s">
         <v>288</v>
       </c>
@@ -5216,7 +5224,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="318" customHeight="1" ht="17.25">
+    <row r="318" spans="1:3" ht="17.25" customHeight="1">
       <c r="A318" s="7" t="s">
         <v>288</v>
       </c>
@@ -5227,7 +5235,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="319" customHeight="1" ht="17.25">
+    <row r="319" spans="1:3" ht="17.25" customHeight="1">
       <c r="A319" s="7" t="s">
         <v>288</v>
       </c>
@@ -5238,7 +5246,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="320" customHeight="1" ht="17.25">
+    <row r="320" spans="1:3" ht="17.25" customHeight="1">
       <c r="A320" s="7" t="s">
         <v>288</v>
       </c>
@@ -5249,7 +5257,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="321" customHeight="1" ht="17.25">
+    <row r="321" spans="1:3" ht="17.25" customHeight="1">
       <c r="A321" s="7" t="s">
         <v>288</v>
       </c>
@@ -5260,7 +5268,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="322" customHeight="1" ht="17.25">
+    <row r="322" spans="1:3" ht="17.25" customHeight="1">
       <c r="A322" s="7" t="s">
         <v>288</v>
       </c>
@@ -5271,7 +5279,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="323" customHeight="1" ht="17.25">
+    <row r="323" spans="1:3" ht="17.25" customHeight="1">
       <c r="A323" s="7" t="s">
         <v>288</v>
       </c>
@@ -5282,7 +5290,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="324" customHeight="1" ht="17.25">
+    <row r="324" spans="1:3" ht="17.25" customHeight="1">
       <c r="A324" s="7" t="s">
         <v>288</v>
       </c>
@@ -5293,7 +5301,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="325" customHeight="1" ht="17.25">
+    <row r="325" spans="1:3" ht="17.25" customHeight="1">
       <c r="A325" s="7" t="s">
         <v>288</v>
       </c>
@@ -5304,7 +5312,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="326" customHeight="1" ht="17.25">
+    <row r="326" spans="1:3" ht="17.25" customHeight="1">
       <c r="A326" s="7" t="s">
         <v>288</v>
       </c>
@@ -5315,7 +5323,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="327" customHeight="1" ht="17.25">
+    <row r="327" spans="1:3" ht="17.25" customHeight="1">
       <c r="A327" s="7" t="s">
         <v>288</v>
       </c>
@@ -5326,7 +5334,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="328" customHeight="1" ht="17.25">
+    <row r="328" spans="1:3" ht="17.25" customHeight="1">
       <c r="A328" s="7" t="s">
         <v>288</v>
       </c>
@@ -5337,7 +5345,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="329" customHeight="1" ht="17.25">
+    <row r="329" spans="1:3" ht="17.25" customHeight="1">
       <c r="A329" s="7" t="s">
         <v>288</v>
       </c>
@@ -5348,7 +5356,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="330" customHeight="1" ht="17.25">
+    <row r="330" spans="1:3" ht="17.25" customHeight="1">
       <c r="A330" s="7" t="s">
         <v>288</v>
       </c>
@@ -5359,7 +5367,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="331" customHeight="1" ht="17.25">
+    <row r="331" spans="1:3" ht="17.25" customHeight="1">
       <c r="A331" s="7" t="s">
         <v>288</v>
       </c>
@@ -5370,7 +5378,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="332" customHeight="1" ht="17.25">
+    <row r="332" spans="1:3" ht="17.25" customHeight="1">
       <c r="A332" s="7" t="s">
         <v>288</v>
       </c>
@@ -5381,7 +5389,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="333" customHeight="1" ht="17.25">
+    <row r="333" spans="1:3" ht="17.25" customHeight="1">
       <c r="A333" s="7" t="s">
         <v>288</v>
       </c>
@@ -5392,17 +5400,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="334" customHeight="1" ht="17.25">
+    <row r="334" spans="1:3" ht="17.25" customHeight="1">
       <c r="A334" s="1"/>
       <c r="B334" s="9"/>
       <c r="C334" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="335" customHeight="1" ht="17.25">
+    <row r="335" spans="1:3" ht="17.25" customHeight="1">
       <c r="A335" s="1"/>
       <c r="B335" s="9"/>
       <c r="C335" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="336" customHeight="1" ht="17.25">
+    <row r="336" spans="1:3" ht="17.25" customHeight="1">
       <c r="A336" s="7" t="s">
         <v>327</v>
       </c>
@@ -5413,7 +5421,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="337" customHeight="1" ht="17.25">
+    <row r="337" spans="1:3" ht="17.25" customHeight="1">
       <c r="A337" s="7" t="s">
         <v>327</v>
       </c>
@@ -5424,7 +5432,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="338" customHeight="1" ht="17.25">
+    <row r="338" spans="1:3" ht="17.25" customHeight="1">
       <c r="A338" s="7" t="s">
         <v>327</v>
       </c>
@@ -5435,7 +5443,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="339" customHeight="1" ht="17.25">
+    <row r="339" spans="1:3" ht="17.25" customHeight="1">
       <c r="A339" s="7" t="s">
         <v>327</v>
       </c>
@@ -5446,7 +5454,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="340" customHeight="1" ht="17.25">
+    <row r="340" spans="1:3" ht="17.25" customHeight="1">
       <c r="A340" s="7" t="s">
         <v>327</v>
       </c>
@@ -5457,7 +5465,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="341" customHeight="1" ht="17.25">
+    <row r="341" spans="1:3" ht="17.25" customHeight="1">
       <c r="A341" s="7" t="s">
         <v>327</v>
       </c>
@@ -5468,7 +5476,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="342" customHeight="1" ht="17.25">
+    <row r="342" spans="1:3" ht="17.25" customHeight="1">
       <c r="A342" s="7" t="s">
         <v>327</v>
       </c>
@@ -5479,7 +5487,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="343" customHeight="1" ht="17.25">
+    <row r="343" spans="1:3" ht="17.25" customHeight="1">
       <c r="A343" s="7" t="s">
         <v>327</v>
       </c>
@@ -5490,7 +5498,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="344" customHeight="1" ht="17.25">
+    <row r="344" spans="1:3" ht="17.25" customHeight="1">
       <c r="A344" s="7" t="s">
         <v>327</v>
       </c>
@@ -5501,7 +5509,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="345" customHeight="1" ht="17.25">
+    <row r="345" spans="1:3" ht="17.25" customHeight="1">
       <c r="A345" s="7" t="s">
         <v>327</v>
       </c>
@@ -5512,7 +5520,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="346" customHeight="1" ht="17.25">
+    <row r="346" spans="1:3" ht="17.25" customHeight="1">
       <c r="A346" s="7" t="s">
         <v>327</v>
       </c>
@@ -5523,7 +5531,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="347" customHeight="1" ht="17.25">
+    <row r="347" spans="1:3" ht="17.25" customHeight="1">
       <c r="A347" s="7" t="s">
         <v>327</v>
       </c>
@@ -5534,7 +5542,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="348" customHeight="1" ht="17.25">
+    <row r="348" spans="1:3" ht="17.25" customHeight="1">
       <c r="A348" s="7" t="s">
         <v>327</v>
       </c>
@@ -5545,7 +5553,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="349" customHeight="1" ht="17.25">
+    <row r="349" spans="1:3" ht="17.25" customHeight="1">
       <c r="A349" s="7" t="s">
         <v>327</v>
       </c>
@@ -5556,7 +5564,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="350" customHeight="1" ht="17.25">
+    <row r="350" spans="1:3" ht="17.25" customHeight="1">
       <c r="A350" s="7" t="s">
         <v>327</v>
       </c>
@@ -5567,7 +5575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="351" customHeight="1" ht="17.25">
+    <row r="351" spans="1:3" ht="17.25" customHeight="1">
       <c r="A351" s="7" t="s">
         <v>327</v>
       </c>
@@ -5578,7 +5586,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="352" customHeight="1" ht="17.25">
+    <row r="352" spans="1:3" ht="17.25" customHeight="1">
       <c r="A352" s="7" t="s">
         <v>327</v>
       </c>
@@ -5589,7 +5597,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="353" customHeight="1" ht="17.25">
+    <row r="353" spans="1:3" ht="17.25" customHeight="1">
       <c r="A353" s="7" t="s">
         <v>327</v>
       </c>
@@ -5600,17 +5608,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="354" customHeight="1" ht="17.25">
+    <row r="354" spans="1:3" ht="17.25" customHeight="1">
       <c r="A354" s="1"/>
       <c r="B354" s="9"/>
       <c r="C354" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="355" customHeight="1" ht="17.25">
+    <row r="355" spans="1:3" ht="17.25" customHeight="1">
       <c r="A355" s="1"/>
       <c r="B355" s="9"/>
       <c r="C355" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="356" customHeight="1" ht="17.25">
+    <row r="356" spans="1:3" ht="17.25" customHeight="1">
       <c r="A356" s="7" t="s">
         <v>346</v>
       </c>
@@ -5621,7 +5629,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="357" customHeight="1" ht="17.25">
+    <row r="357" spans="1:3" ht="17.25" customHeight="1">
       <c r="A357" s="7" t="s">
         <v>346</v>
       </c>
@@ -5632,7 +5640,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="358" customHeight="1" ht="17.25">
+    <row r="358" spans="1:3" ht="17.25" customHeight="1">
       <c r="A358" s="7" t="s">
         <v>346</v>
       </c>
@@ -5643,7 +5651,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="359" customHeight="1" ht="17.25">
+    <row r="359" spans="1:3" ht="17.25" customHeight="1">
       <c r="A359" s="7" t="s">
         <v>346</v>
       </c>
@@ -5654,7 +5662,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="360" customHeight="1" ht="17.25">
+    <row r="360" spans="1:3" ht="17.25" customHeight="1">
       <c r="A360" s="7" t="s">
         <v>346</v>
       </c>
@@ -5665,7 +5673,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="361" customHeight="1" ht="17.25">
+    <row r="361" spans="1:3" ht="17.25" customHeight="1">
       <c r="A361" s="7" t="s">
         <v>346</v>
       </c>
@@ -5676,7 +5684,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="362" customHeight="1" ht="17.25">
+    <row r="362" spans="1:3" ht="17.25" customHeight="1">
       <c r="A362" s="7" t="s">
         <v>346</v>
       </c>
@@ -5687,7 +5695,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="363" customHeight="1" ht="17.25">
+    <row r="363" spans="1:3" ht="17.25" customHeight="1">
       <c r="A363" s="7" t="s">
         <v>346</v>
       </c>
@@ -5698,7 +5706,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="364" customHeight="1" ht="17.25">
+    <row r="364" spans="1:3" ht="17.25" customHeight="1">
       <c r="A364" s="7" t="s">
         <v>346</v>
       </c>
@@ -5709,7 +5717,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="365" customHeight="1" ht="17.25">
+    <row r="365" spans="1:3" ht="17.25" customHeight="1">
       <c r="A365" s="7" t="s">
         <v>346</v>
       </c>
@@ -5720,7 +5728,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="366" customHeight="1" ht="17.25">
+    <row r="366" spans="1:3" ht="17.25" customHeight="1">
       <c r="A366" s="7" t="s">
         <v>346</v>
       </c>
@@ -5731,7 +5739,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="367" customHeight="1" ht="17.25">
+    <row r="367" spans="1:3" ht="17.25" customHeight="1">
       <c r="A367" s="7" t="s">
         <v>346</v>
       </c>
@@ -5742,7 +5750,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="368" customHeight="1" ht="17.25">
+    <row r="368" spans="1:3" ht="17.25" customHeight="1">
       <c r="A368" s="7" t="s">
         <v>346</v>
       </c>
@@ -5753,7 +5761,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="369" customHeight="1" ht="17.25">
+    <row r="369" spans="1:3" ht="17.25" customHeight="1">
       <c r="A369" s="7" t="s">
         <v>346</v>
       </c>
@@ -5764,7 +5772,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="370" customHeight="1" ht="17.25">
+    <row r="370" spans="1:3" ht="17.25" customHeight="1">
       <c r="A370" s="7" t="s">
         <v>346</v>
       </c>
@@ -5775,7 +5783,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="371" customHeight="1" ht="17.25">
+    <row r="371" spans="1:3" ht="17.25" customHeight="1">
       <c r="A371" s="7" t="s">
         <v>346</v>
       </c>
@@ -5786,7 +5794,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="372" customHeight="1" ht="17.25">
+    <row r="372" spans="1:3" ht="17.25" customHeight="1">
       <c r="A372" s="7" t="s">
         <v>346</v>
       </c>
@@ -5797,7 +5805,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="373" customHeight="1" ht="17.25">
+    <row r="373" spans="1:3" ht="17.25" customHeight="1">
       <c r="A373" s="7" t="s">
         <v>346</v>
       </c>
@@ -5808,7 +5816,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="374" customHeight="1" ht="17.25">
+    <row r="374" spans="1:3" ht="17.25" customHeight="1">
       <c r="A374" s="7" t="s">
         <v>346</v>
       </c>
@@ -5819,7 +5827,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="375" customHeight="1" ht="17.25">
+    <row r="375" spans="1:3" ht="17.25" customHeight="1">
       <c r="A375" s="7" t="s">
         <v>346</v>
       </c>
@@ -5830,7 +5838,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="376" customHeight="1" ht="17.25">
+    <row r="376" spans="1:3" ht="17.25" customHeight="1">
       <c r="A376" s="7" t="s">
         <v>346</v>
       </c>
@@ -5841,7 +5849,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="377" customHeight="1" ht="17.25">
+    <row r="377" spans="1:3" ht="17.25" customHeight="1">
       <c r="A377" s="7" t="s">
         <v>346</v>
       </c>
@@ -5852,7 +5860,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="378" customHeight="1" ht="17.25">
+    <row r="378" spans="1:3" ht="17.25" customHeight="1">
       <c r="A378" s="7" t="s">
         <v>346</v>
       </c>
@@ -5863,7 +5871,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="379" customHeight="1" ht="17.25">
+    <row r="379" spans="1:3" ht="17.25" customHeight="1">
       <c r="A379" s="7" t="s">
         <v>346</v>
       </c>
@@ -5874,7 +5882,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="380" customHeight="1" ht="17.25">
+    <row r="380" spans="1:3" ht="17.25" customHeight="1">
       <c r="A380" s="7" t="s">
         <v>346</v>
       </c>
@@ -5885,7 +5893,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="381" customHeight="1" ht="17.25">
+    <row r="381" spans="1:3" ht="17.25" customHeight="1">
       <c r="A381" s="7" t="s">
         <v>346</v>
       </c>
@@ -5896,7 +5904,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="382" customHeight="1" ht="17.25">
+    <row r="382" spans="1:3" ht="17.25" customHeight="1">
       <c r="A382" s="7" t="s">
         <v>346</v>
       </c>
@@ -5907,7 +5915,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="383" customHeight="1" ht="17.25">
+    <row r="383" spans="1:3" ht="17.25" customHeight="1">
       <c r="A383" s="7" t="s">
         <v>346</v>
       </c>
@@ -5918,7 +5926,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="384" customHeight="1" ht="17.25">
+    <row r="384" spans="1:3" ht="17.25" customHeight="1">
       <c r="A384" s="7" t="s">
         <v>346</v>
       </c>
@@ -5929,7 +5937,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="385" customHeight="1" ht="17.25">
+    <row r="385" spans="1:3" ht="17.25" customHeight="1">
       <c r="A385" s="7" t="s">
         <v>346</v>
       </c>
@@ -5940,7 +5948,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="386" customHeight="1" ht="17.25">
+    <row r="386" spans="1:3" ht="17.25" customHeight="1">
       <c r="A386" s="7" t="s">
         <v>346</v>
       </c>
@@ -5951,7 +5959,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="387" customHeight="1" ht="17.25">
+    <row r="387" spans="1:3" ht="17.25" customHeight="1">
       <c r="A387" s="7" t="s">
         <v>346</v>
       </c>
@@ -5962,7 +5970,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="388" customHeight="1" ht="17.25">
+    <row r="388" spans="1:3" ht="17.25" customHeight="1">
       <c r="A388" s="7" t="s">
         <v>346</v>
       </c>
@@ -5973,7 +5981,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="389" customHeight="1" ht="17.25">
+    <row r="389" spans="1:3" ht="17.25" customHeight="1">
       <c r="A389" s="7" t="s">
         <v>346</v>
       </c>
@@ -5984,7 +5992,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="390" customHeight="1" ht="17.25">
+    <row r="390" spans="1:3" ht="17.25" customHeight="1">
       <c r="A390" s="7" t="s">
         <v>346</v>
       </c>
@@ -5995,7 +6003,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="391" customHeight="1" ht="17.25">
+    <row r="391" spans="1:3" ht="17.25" customHeight="1">
       <c r="A391" s="7" t="s">
         <v>346</v>
       </c>
@@ -6006,7 +6014,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="392" customHeight="1" ht="17.25">
+    <row r="392" spans="1:3" ht="17.25" customHeight="1">
       <c r="A392" s="7" t="s">
         <v>346</v>
       </c>
@@ -6017,7 +6025,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="393" customHeight="1" ht="17.25">
+    <row r="393" spans="1:3" ht="17.25" customHeight="1">
       <c r="A393" s="7" t="s">
         <v>346</v>
       </c>
@@ -6028,7 +6036,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="394" customHeight="1" ht="17.25">
+    <row r="394" spans="1:3" ht="17.25" customHeight="1">
       <c r="A394" s="7" t="s">
         <v>346</v>
       </c>
@@ -6039,7 +6047,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="395" customHeight="1" ht="17.25">
+    <row r="395" spans="1:3" ht="17.25" customHeight="1">
       <c r="A395" s="7" t="s">
         <v>346</v>
       </c>
@@ -6050,7 +6058,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="396" customHeight="1" ht="17.25">
+    <row r="396" spans="1:3" ht="17.25" customHeight="1">
       <c r="A396" s="7" t="s">
         <v>346</v>
       </c>
@@ -6061,7 +6069,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="397" customHeight="1" ht="17.25">
+    <row r="397" spans="1:3" ht="17.25" customHeight="1">
       <c r="A397" s="7" t="s">
         <v>346</v>
       </c>
@@ -6072,7 +6080,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="398" customHeight="1" ht="17.25">
+    <row r="398" spans="1:3" ht="17.25" customHeight="1">
       <c r="A398" s="7" t="s">
         <v>346</v>
       </c>
@@ -6083,7 +6091,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="399" customHeight="1" ht="17.25">
+    <row r="399" spans="1:3" ht="17.25" customHeight="1">
       <c r="A399" s="7" t="s">
         <v>346</v>
       </c>
@@ -6094,17 +6102,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="400" customHeight="1" ht="17.25">
+    <row r="400" spans="1:3" ht="17.25" customHeight="1">
       <c r="A400" s="1"/>
       <c r="B400" s="9"/>
       <c r="C400" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="401" customHeight="1" ht="17.25">
+    <row r="401" spans="1:3" ht="17.25" customHeight="1">
       <c r="A401" s="1"/>
       <c r="B401" s="9"/>
       <c r="C401" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="402" customHeight="1" ht="17.25">
+    <row r="402" spans="1:3" ht="17.25" customHeight="1">
       <c r="A402" s="7" t="s">
         <v>390</v>
       </c>
@@ -6115,7 +6123,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="403" customHeight="1" ht="17.25">
+    <row r="403" spans="1:3" ht="17.25" customHeight="1">
       <c r="A403" s="7" t="s">
         <v>390</v>
       </c>
@@ -6126,7 +6134,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="404" customHeight="1" ht="17.25">
+    <row r="404" spans="1:3" ht="17.25" customHeight="1">
       <c r="A404" s="7" t="s">
         <v>390</v>
       </c>
@@ -6137,7 +6145,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="405" customHeight="1" ht="17.25">
+    <row r="405" spans="1:3" ht="17.25" customHeight="1">
       <c r="A405" s="7" t="s">
         <v>390</v>
       </c>
@@ -6148,7 +6156,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="406" customHeight="1" ht="17.25">
+    <row r="406" spans="1:3" ht="17.25" customHeight="1">
       <c r="A406" s="7" t="s">
         <v>390</v>
       </c>
@@ -6159,7 +6167,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="407" customHeight="1" ht="17.25">
+    <row r="407" spans="1:3" ht="17.25" customHeight="1">
       <c r="A407" s="7" t="s">
         <v>390</v>
       </c>
@@ -6170,17 +6178,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="408" customHeight="1" ht="17.25">
+    <row r="408" spans="1:3" ht="17.25" customHeight="1">
       <c r="A408" s="1"/>
       <c r="B408" s="9"/>
       <c r="C408" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="409" customHeight="1" ht="17.25">
+    <row r="409" spans="1:3" ht="17.25" customHeight="1">
       <c r="A409" s="1"/>
       <c r="B409" s="9"/>
       <c r="C409" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="410" customHeight="1" ht="17.25">
+    <row r="410" spans="1:3" ht="17.25" customHeight="1">
       <c r="A410" s="7" t="s">
         <v>396</v>
       </c>
@@ -6191,7 +6199,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="411" customHeight="1" ht="17.25">
+    <row r="411" spans="1:3" ht="17.25" customHeight="1">
       <c r="A411" s="7" t="s">
         <v>396</v>
       </c>
@@ -6202,7 +6210,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="412" customHeight="1" ht="17.25">
+    <row r="412" spans="1:3" ht="17.25" customHeight="1">
       <c r="A412" s="7" t="s">
         <v>396</v>
       </c>
@@ -6213,7 +6221,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="413" customHeight="1" ht="17.25">
+    <row r="413" spans="1:3" ht="17.25" customHeight="1">
       <c r="A413" s="7" t="s">
         <v>396</v>
       </c>
@@ -6224,7 +6232,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="414" customHeight="1" ht="17.25">
+    <row r="414" spans="1:3" ht="17.25" customHeight="1">
       <c r="A414" s="7" t="s">
         <v>396</v>
       </c>
@@ -6235,7 +6243,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="415" customHeight="1" ht="17.25">
+    <row r="415" spans="1:3" ht="17.25" customHeight="1">
       <c r="A415" s="7" t="s">
         <v>396</v>
       </c>
@@ -6246,7 +6254,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="416" customHeight="1" ht="17.25">
+    <row r="416" spans="1:3" ht="17.25" customHeight="1">
       <c r="A416" s="7" t="s">
         <v>396</v>
       </c>
@@ -6257,7 +6265,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="417" customHeight="1" ht="17.25">
+    <row r="417" spans="1:3" ht="17.25" customHeight="1">
       <c r="A417" s="7" t="s">
         <v>396</v>
       </c>
@@ -6268,7 +6276,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="418" customHeight="1" ht="17.25">
+    <row r="418" spans="1:3" ht="17.25" customHeight="1">
       <c r="A418" s="7" t="s">
         <v>396</v>
       </c>
@@ -6279,7 +6287,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="419" customHeight="1" ht="17.25">
+    <row r="419" spans="1:3" ht="17.25" customHeight="1">
       <c r="A419" s="7" t="s">
         <v>396</v>
       </c>
@@ -6290,7 +6298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="420" customHeight="1" ht="17.25">
+    <row r="420" spans="1:3" ht="17.25" customHeight="1">
       <c r="A420" s="7" t="s">
         <v>396</v>
       </c>
@@ -6301,7 +6309,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="421" customHeight="1" ht="17.25">
+    <row r="421" spans="1:3" ht="17.25" customHeight="1">
       <c r="A421" s="7" t="s">
         <v>396</v>
       </c>
@@ -6312,7 +6320,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="422" customHeight="1" ht="17.25">
+    <row r="422" spans="1:3" ht="17.25" customHeight="1">
       <c r="A422" s="7" t="s">
         <v>396</v>
       </c>
@@ -6323,7 +6331,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="423" customHeight="1" ht="17.25">
+    <row r="423" spans="1:3" ht="17.25" customHeight="1">
       <c r="A423" s="7" t="s">
         <v>396</v>
       </c>
@@ -6334,7 +6342,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="424" customHeight="1" ht="17.25">
+    <row r="424" spans="1:3" ht="17.25" customHeight="1">
       <c r="A424" s="7" t="s">
         <v>396</v>
       </c>
@@ -6345,7 +6353,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="425" customHeight="1" ht="17.25">
+    <row r="425" spans="1:3" ht="17.25" customHeight="1">
       <c r="A425" s="7" t="s">
         <v>396</v>
       </c>
@@ -6356,7 +6364,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="426" customHeight="1" ht="17.25">
+    <row r="426" spans="1:3" ht="17.25" customHeight="1">
       <c r="A426" s="7" t="s">
         <v>396</v>
       </c>
@@ -6367,7 +6375,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="427" customHeight="1" ht="17.25">
+    <row r="427" spans="1:3" ht="17.25" customHeight="1">
       <c r="A427" s="7" t="s">
         <v>396</v>
       </c>
@@ -6378,7 +6386,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="428" customHeight="1" ht="17.25">
+    <row r="428" spans="1:3" ht="17.25" customHeight="1">
       <c r="A428" s="7" t="s">
         <v>396</v>
       </c>
@@ -6389,7 +6397,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="429" customHeight="1" ht="17.25">
+    <row r="429" spans="1:3" ht="17.25" customHeight="1">
       <c r="A429" s="7" t="s">
         <v>396</v>
       </c>
@@ -6400,7 +6408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="430" customHeight="1" ht="17.25">
+    <row r="430" spans="1:3" ht="17.25" customHeight="1">
       <c r="A430" s="7" t="s">
         <v>396</v>
       </c>
@@ -6411,7 +6419,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="431" customHeight="1" ht="17.25">
+    <row r="431" spans="1:3" ht="17.25" customHeight="1">
       <c r="A431" s="7" t="s">
         <v>396</v>
       </c>
@@ -6422,7 +6430,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="432" customHeight="1" ht="17.25">
+    <row r="432" spans="1:3" ht="17.25" customHeight="1">
       <c r="A432" s="7" t="s">
         <v>396</v>
       </c>
@@ -6433,7 +6441,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="433" customHeight="1" ht="17.25">
+    <row r="433" spans="1:3" ht="17.25" customHeight="1">
       <c r="A433" s="7" t="s">
         <v>396</v>
       </c>
@@ -6444,7 +6452,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="434" customHeight="1" ht="17.25">
+    <row r="434" spans="1:3" ht="17.25" customHeight="1">
       <c r="A434" s="7" t="s">
         <v>396</v>
       </c>
@@ -6455,7 +6463,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="435" customHeight="1" ht="17.25">
+    <row r="435" spans="1:3" ht="17.25" customHeight="1">
       <c r="A435" s="7" t="s">
         <v>396</v>
       </c>
@@ -6466,7 +6474,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="436" customHeight="1" ht="17.25">
+    <row r="436" spans="1:3" ht="17.25" customHeight="1">
       <c r="A436" s="7" t="s">
         <v>396</v>
       </c>
@@ -6477,7 +6485,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="437" customHeight="1" ht="17.25">
+    <row r="437" spans="1:3" ht="17.25" customHeight="1">
       <c r="A437" s="7" t="s">
         <v>396</v>
       </c>
@@ -6488,7 +6496,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="438" customHeight="1" ht="17.25">
+    <row r="438" spans="1:3" ht="17.25" customHeight="1">
       <c r="A438" s="7" t="s">
         <v>396</v>
       </c>
@@ -6499,7 +6507,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="439" customHeight="1" ht="17.25">
+    <row r="439" spans="1:3" ht="17.25" customHeight="1">
       <c r="A439" s="7" t="s">
         <v>396</v>
       </c>
@@ -6510,7 +6518,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="440" customHeight="1" ht="17.25">
+    <row r="440" spans="1:3" ht="17.25" customHeight="1">
       <c r="A440" s="7" t="s">
         <v>396</v>
       </c>
@@ -6521,7 +6529,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="441" customHeight="1" ht="17.25">
+    <row r="441" spans="1:3" ht="17.25" customHeight="1">
       <c r="A441" s="7" t="s">
         <v>396</v>
       </c>
@@ -6532,7 +6540,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="442" customHeight="1" ht="17.25">
+    <row r="442" spans="1:3" ht="17.25" customHeight="1">
       <c r="A442" s="7" t="s">
         <v>396</v>
       </c>
@@ -6543,7 +6551,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="443" customHeight="1" ht="17.25">
+    <row r="443" spans="1:3" ht="17.25" customHeight="1">
       <c r="A443" s="7" t="s">
         <v>396</v>
       </c>
@@ -6554,7 +6562,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="444" customHeight="1" ht="17.25">
+    <row r="444" spans="1:3" ht="17.25" customHeight="1">
       <c r="A444" s="7" t="s">
         <v>396</v>
       </c>
@@ -6565,7 +6573,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="445" customHeight="1" ht="17.25">
+    <row r="445" spans="1:3" ht="17.25" customHeight="1">
       <c r="A445" s="7" t="s">
         <v>396</v>
       </c>
@@ -6576,7 +6584,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="446" customHeight="1" ht="17.25">
+    <row r="446" spans="1:3" ht="17.25" customHeight="1">
       <c r="A446" s="7" t="s">
         <v>396</v>
       </c>
@@ -6587,7 +6595,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="447" customHeight="1" ht="17.25">
+    <row r="447" spans="1:3" ht="17.25" customHeight="1">
       <c r="A447" s="7" t="s">
         <v>396</v>
       </c>
@@ -6598,7 +6606,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="448" customHeight="1" ht="17.25">
+    <row r="448" spans="1:3" ht="17.25" customHeight="1">
       <c r="A448" s="7" t="s">
         <v>396</v>
       </c>
@@ -6609,7 +6617,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="449" customHeight="1" ht="17.25">
+    <row r="449" spans="1:3" ht="17.25" customHeight="1">
       <c r="A449" s="7" t="s">
         <v>396</v>
       </c>
@@ -6620,7 +6628,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="450" customHeight="1" ht="17.25">
+    <row r="450" spans="1:3" ht="17.25" customHeight="1">
       <c r="A450" s="7" t="s">
         <v>396</v>
       </c>
@@ -6631,7 +6639,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="451" customHeight="1" ht="17.25">
+    <row r="451" spans="1:3" ht="17.25" customHeight="1">
       <c r="A451" s="7" t="s">
         <v>396</v>
       </c>
@@ -6642,7 +6650,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="452" customHeight="1" ht="17.25">
+    <row r="452" spans="1:3" ht="17.25" customHeight="1">
       <c r="A452" s="7" t="s">
         <v>396</v>
       </c>
@@ -6653,7 +6661,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="453" customHeight="1" ht="17.25">
+    <row r="453" spans="1:3" ht="17.25" customHeight="1">
       <c r="A453" s="7" t="s">
         <v>396</v>
       </c>
@@ -6664,7 +6672,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="454" customHeight="1" ht="17.25">
+    <row r="454" spans="1:3" ht="17.25" customHeight="1">
       <c r="A454" s="7" t="s">
         <v>396</v>
       </c>
@@ -6675,7 +6683,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="455" customHeight="1" ht="17.25">
+    <row r="455" spans="1:3" ht="17.25" customHeight="1">
       <c r="A455" s="7" t="s">
         <v>396</v>
       </c>
@@ -6686,7 +6694,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="456" customHeight="1" ht="17.25">
+    <row r="456" spans="1:3" ht="17.25" customHeight="1">
       <c r="A456" s="7" t="s">
         <v>396</v>
       </c>
@@ -6697,7 +6705,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="457" customHeight="1" ht="17.25">
+    <row r="457" spans="1:3" ht="17.25" customHeight="1">
       <c r="A457" s="7" t="s">
         <v>396</v>
       </c>
@@ -6708,7 +6716,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="458" customHeight="1" ht="17.25">
+    <row r="458" spans="1:3" ht="17.25" customHeight="1">
       <c r="A458" s="7" t="s">
         <v>396</v>
       </c>
@@ -6719,7 +6727,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="459" customHeight="1" ht="17.25">
+    <row r="459" spans="1:3" ht="17.25" customHeight="1">
       <c r="A459" s="7" t="s">
         <v>396</v>
       </c>
@@ -6730,7 +6738,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="460" customHeight="1" ht="17.25">
+    <row r="460" spans="1:3" ht="17.25" customHeight="1">
       <c r="A460" s="7" t="s">
         <v>396</v>
       </c>
@@ -6741,7 +6749,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="461" customHeight="1" ht="17.25">
+    <row r="461" spans="1:3" ht="17.25" customHeight="1">
       <c r="A461" s="7" t="s">
         <v>396</v>
       </c>
@@ -6752,7 +6760,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="462" customHeight="1" ht="17.25">
+    <row r="462" spans="1:3" ht="17.25" customHeight="1">
       <c r="A462" s="7" t="s">
         <v>396</v>
       </c>
@@ -6763,7 +6771,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="463" customHeight="1" ht="17.25">
+    <row r="463" spans="1:3" ht="17.25" customHeight="1">
       <c r="A463" s="7" t="s">
         <v>396</v>
       </c>
@@ -6774,7 +6782,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="464" customHeight="1" ht="17.25">
+    <row r="464" spans="1:3" ht="17.25" customHeight="1">
       <c r="A464" s="7" t="s">
         <v>396</v>
       </c>
@@ -6785,7 +6793,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="465" customHeight="1" ht="17.25">
+    <row r="465" spans="1:3" ht="17.25" customHeight="1">
       <c r="A465" s="7" t="s">
         <v>396</v>
       </c>
@@ -6796,7 +6804,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="466" customHeight="1" ht="17.25">
+    <row r="466" spans="1:3" ht="17.25" customHeight="1">
       <c r="A466" s="7" t="s">
         <v>396</v>
       </c>
@@ -6807,7 +6815,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="467" customHeight="1" ht="17.25">
+    <row r="467" spans="1:3" ht="17.25" customHeight="1">
       <c r="A467" s="7" t="s">
         <v>396</v>
       </c>
@@ -6818,7 +6826,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="468" customHeight="1" ht="17.25">
+    <row r="468" spans="1:3" ht="17.25" customHeight="1">
       <c r="A468" s="7" t="s">
         <v>396</v>
       </c>
@@ -6829,7 +6837,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="469" customHeight="1" ht="17.25">
+    <row r="469" spans="1:3" ht="17.25" customHeight="1">
       <c r="A469" s="7" t="s">
         <v>396</v>
       </c>
@@ -6840,17 +6848,17 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="470" customHeight="1" ht="17.25">
+    <row r="470" spans="1:3" ht="17.25" customHeight="1">
       <c r="A470" s="1"/>
       <c r="B470" s="9"/>
       <c r="C470" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="471" customHeight="1" ht="17.25">
+    <row r="471" spans="1:3" ht="17.25" customHeight="1">
       <c r="A471" s="7"/>
       <c r="B471" s="9"/>
       <c r="C471" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="472" customHeight="1" ht="17.25">
+    <row r="472" spans="1:3" ht="17.25" customHeight="1">
       <c r="A472" s="7" t="s">
         <v>456</v>
       </c>
@@ -6861,7 +6869,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="473" customHeight="1" ht="17.25">
+    <row r="473" spans="1:3" ht="17.25" customHeight="1">
       <c r="A473" s="7" t="s">
         <v>456</v>
       </c>
@@ -6872,7 +6880,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="474" customHeight="1" ht="17.25">
+    <row r="474" spans="1:3" ht="17.25" customHeight="1">
       <c r="A474" s="7" t="s">
         <v>456</v>
       </c>
@@ -6883,7 +6891,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="475" customHeight="1" ht="17.25">
+    <row r="475" spans="1:3" ht="17.25" customHeight="1">
       <c r="A475" s="7" t="s">
         <v>456</v>
       </c>
@@ -6894,7 +6902,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="476" customHeight="1" ht="17.25">
+    <row r="476" spans="1:3" ht="17.25" customHeight="1">
       <c r="A476" s="7" t="s">
         <v>456</v>
       </c>
@@ -6905,7 +6913,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="477" customHeight="1" ht="17.25">
+    <row r="477" spans="1:3" ht="17.25" customHeight="1">
       <c r="A477" s="7" t="s">
         <v>456</v>
       </c>
@@ -6916,7 +6924,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="478" customHeight="1" ht="17.25">
+    <row r="478" spans="1:3" ht="17.25" customHeight="1">
       <c r="A478" s="7" t="s">
         <v>456</v>
       </c>
@@ -6927,7 +6935,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="479" customHeight="1" ht="17.25">
+    <row r="479" spans="1:3" ht="17.25" customHeight="1">
       <c r="A479" s="7" t="s">
         <v>456</v>
       </c>
@@ -6938,7 +6946,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="480" customHeight="1" ht="17.25">
+    <row r="480" spans="1:3" ht="17.25" customHeight="1">
       <c r="A480" s="7" t="s">
         <v>456</v>
       </c>
@@ -6949,7 +6957,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="481" customHeight="1" ht="17.25">
+    <row r="481" spans="1:3" ht="17.25" customHeight="1">
       <c r="A481" s="7" t="s">
         <v>456</v>
       </c>

</xml_diff>